<commit_message>
Day 04 Learning Excel
</commit_message>
<xml_diff>
--- a/Day 01.xlsx
+++ b/Day 01.xlsx
@@ -9,22 +9,24 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet4" sheetId="5" r:id="rId4"/>
-    <sheet name="Sheet8" sheetId="9" r:id="rId5"/>
-    <sheet name="Sheet5" sheetId="7" r:id="rId6"/>
+    <sheet name="Sheet5" sheetId="7" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="9" r:id="rId6"/>
+    <sheet name="Sheet7" sheetId="11" r:id="rId7"/>
+    <sheet name="Sheet8" sheetId="12" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet3!$A$1:$C$11</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="6" r:id="rId7"/>
+    <pivotCache cacheId="5" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="87">
   <si>
     <t>Alex</t>
   </si>
@@ -245,6 +247,57 @@
   </si>
   <si>
     <t>(All)</t>
+  </si>
+  <si>
+    <t>Bilal</t>
+  </si>
+  <si>
+    <t>Ayesha</t>
+  </si>
+  <si>
+    <t>Peshawar</t>
+  </si>
+  <si>
+    <t>Attendance(%)</t>
+  </si>
+  <si>
+    <t>Bonus</t>
+  </si>
+  <si>
+    <t>City Type</t>
+  </si>
+  <si>
+    <t>Top Performer</t>
+  </si>
+  <si>
+    <t>ahmed khan</t>
+  </si>
+  <si>
+    <t>SARA ALI</t>
+  </si>
+  <si>
+    <t>AYESHA KHAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  bilal ahmed</t>
+  </si>
+  <si>
+    <t>lahore</t>
+  </si>
+  <si>
+    <t>islamabad</t>
+  </si>
+  <si>
+    <t>Clean Name</t>
+  </si>
+  <si>
+    <t>Clean City</t>
+  </si>
+  <si>
+    <t>Trimmed Name</t>
+  </si>
+  <si>
+    <t>Unknown</t>
   </si>
 </sst>
 </file>
@@ -283,7 +336,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -323,6 +376,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -391,7 +450,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -400,6 +459,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -409,13 +475,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -474,7 +534,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -564,7 +623,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -849,7 +907,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -940,7 +997,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -1225,7 +1281,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1601,7 +1656,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3424,7 +3478,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="umer" refreshedDate="46117.668395833331" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="12">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="umer" refreshedDate="46117.881428125002" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="12">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:D13" sheet="Sheet5"/>
   </cacheSource>
@@ -3541,7 +3595,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:D8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="4">
     <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
@@ -3929,11 +3983,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="10"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -4475,62 +4529,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="9">
         <v>85</v>
       </c>
-      <c r="C2" s="12" t="str">
+      <c r="C2" s="9" t="str">
         <f>VLOOKUP(A2,$J$2:$L$6,2,0)</f>
         <v>Ahmed</v>
       </c>
-      <c r="D2" s="12" t="str">
+      <c r="D2" s="9" t="str">
         <f>VLOOKUP(A2,$J$2:$L$6,3,0)</f>
         <v>A</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="9" t="s">
         <v>45</v>
       </c>
     </row>
@@ -4566,33 +4620,33 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="9">
         <v>91</v>
       </c>
-      <c r="C4" s="12" t="str">
+      <c r="C4" s="9" t="str">
         <f>VLOOKUP(A4,$J$2:$L$6,2,0)</f>
         <v>Hamza</v>
       </c>
-      <c r="D4" s="12" t="str">
+      <c r="D4" s="9" t="str">
         <f>VLOOKUP(A4,$J$2:$L$6,3,0)</f>
         <v>A+</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="L4" s="9" t="s">
         <v>47</v>
       </c>
     </row>
@@ -4628,33 +4682,33 @@
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="9">
         <v>78</v>
       </c>
-      <c r="C6" s="12" t="str">
+      <c r="C6" s="9" t="str">
         <f>VLOOKUP(A6,$J$2:$L$6,2,0)</f>
         <v>Usman</v>
       </c>
-      <c r="D6" s="12" t="str">
+      <c r="D6" s="9" t="str">
         <f>VLOOKUP(A6,$J$2:$L$6,3,0)</f>
         <v>B+</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="J6" s="12" t="s">
+      <c r="J6" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="K6" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="L6" s="9" t="s">
         <v>49</v>
       </c>
     </row>
@@ -4678,6 +4732,204 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="9">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="2">
+        <v>3800</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="9">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="2">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="9">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2">
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="9">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="2">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="9">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="2">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="9">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="2">
+        <v>4100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4688,7 +4940,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="10" t="s">
         <v>60</v>
       </c>
       <c r="B1" t="s">
@@ -4696,15 +4948,15 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="10" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>65</v>
       </c>
       <c r="B4" t="s">
@@ -4718,59 +4970,310 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="12">
         <v>5400</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="12">
         <v>7400</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="12">
         <v>12800</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="12">
         <v>4300</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="12">
         <v>6900</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="12">
         <v>11200</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="12">
         <v>3700</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="12">
         <v>6700</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="12">
         <v>10400</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="12">
         <v>13400</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="12">
         <v>21000</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="12">
         <v>34400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="9">
+        <v>3500</v>
+      </c>
+      <c r="C2" s="9">
+        <v>95</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="9" t="str">
+        <f>IF(AND(B2&gt;2500,C2&gt;90),"Yes - Bonus!","No Bonus")</f>
+        <v>Yes - Bonus!</v>
+      </c>
+      <c r="F2" s="9" t="str">
+        <f>IF(OR(D2="Lahore",D2="Karachi"),"Major City","Other City")</f>
+        <v>Major City</v>
+      </c>
+      <c r="G2" s="9" t="str">
+        <f>IF(AND(B2&gt;3000,C2&gt;90,D2="Lahore"),"Star!","Regular")</f>
+        <v>Star!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2800</v>
+      </c>
+      <c r="C3" s="2">
+        <v>88</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="5" t="str">
+        <f t="shared" ref="E3:E9" si="0">IF(AND(B3&gt;2500,C3&gt;90),"Yes - Bonus!","No Bonus")</f>
+        <v>No Bonus</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <f t="shared" ref="F3:F9" si="1">IF(OR(D3="Lahore",D3="Karachi"),"Major City","Other City")</f>
+        <v>Major City</v>
+      </c>
+      <c r="G3" s="2" t="str">
+        <f t="shared" ref="G3:G9" si="2">IF(AND(B3&gt;3000,C3&gt;90,D3="Lahore"),"Star!","Regular")</f>
+        <v>Regular</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="9">
+        <v>4200</v>
+      </c>
+      <c r="C4" s="9">
+        <v>92</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>Yes - Bonus!</v>
+      </c>
+      <c r="F4" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v>Other City</v>
+      </c>
+      <c r="G4" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v>Regular</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="2">
+        <v>3100</v>
+      </c>
+      <c r="C5" s="2">
+        <v>78</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>No Bonus</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>Major City</v>
+      </c>
+      <c r="G5" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>Regular</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="9">
+        <v>2500</v>
+      </c>
+      <c r="C6" s="9">
+        <v>96</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>No Bonus</v>
+      </c>
+      <c r="F6" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v>Other City</v>
+      </c>
+      <c r="G6" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v>Regular</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="2">
+        <v>3800</v>
+      </c>
+      <c r="C7" s="2">
+        <v>85</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>No Bonus</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>Major City</v>
+      </c>
+      <c r="G7" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>Regular</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="9">
+        <v>4500</v>
+      </c>
+      <c r="C8" s="9">
+        <v>91</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>Yes - Bonus!</v>
+      </c>
+      <c r="F8" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v>Major City</v>
+      </c>
+      <c r="G8" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v>Star!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" s="2">
+        <v>2200</v>
+      </c>
+      <c r="C9" s="2">
+        <v>94</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>No Bonus</v>
+      </c>
+      <c r="F9" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>Other City</v>
+      </c>
+      <c r="G9" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>Regular</v>
       </c>
     </row>
   </sheetData>
@@ -4778,197 +5281,221 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1" s="11" t="s">
+    <row r="1" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="11" t="s">
+      <c r="C1" s="8" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="12">
+      <c r="D1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="16">
         <v>2500</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D2" s="16" t="str">
+        <f>PROPER(A2)</f>
+        <v>Ahmed Khan</v>
+      </c>
+      <c r="E2" s="16" t="str">
+        <f>PROPER(B2)</f>
+        <v>Lahore</v>
+      </c>
+      <c r="F2" s="16" t="str">
+        <f>TRIM(PROPER(A2))</f>
+        <v>Ahmed Khan</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="C3" s="2">
         <v>3800</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="B4" s="12" t="s">
+      <c r="D3" s="2" t="str">
+        <f t="shared" ref="D3:D9" si="0">PROPER(A3)</f>
+        <v>Sara Ali</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <f t="shared" ref="E3:E9" si="1">PROPER(B3)</f>
+        <v>Karachi</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <f t="shared" ref="F3:F9" si="2">TRIM(PROPER(A3))</f>
+        <v>Sara Ali</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="12">
+      <c r="C4" s="16">
         <v>1900</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D4" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>Unknown</v>
+      </c>
+      <c r="E4" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v>Islamabad</v>
+      </c>
+      <c r="F4" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v>Unknown</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>43</v>
+        <v>86</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="2">
+        <v>81</v>
+      </c>
+      <c r="C5" s="2">
         <v>4200</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="12" t="s">
+      <c r="D5" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>Unknown</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>Lahore</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>Unknown</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="12">
+      <c r="C6" s="16">
         <v>2100</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D6" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>Unknown</v>
+      </c>
+      <c r="E6" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v>Karachi</v>
+      </c>
+      <c r="F6" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v>Unknown</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="2">
+        <v>81</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2500</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>Unknown</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>Lahore</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>Unknown</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" s="16">
         <v>3300</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="12">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D8" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v>Ayesha Khan</v>
+      </c>
+      <c r="E8" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v>Islamabad</v>
+      </c>
+      <c r="F8" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v>Ayesha Khan</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="2">
+      <c r="C9" s="2">
         <v>2900</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="12">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="2">
-        <v>2700</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="12">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" s="2">
-        <v>4100</v>
+      <c r="D9" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">  Bilal Ahmed</v>
+      </c>
+      <c r="E9" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>Karachi</v>
+      </c>
+      <c r="F9" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>Bilal Ahmed</v>
       </c>
     </row>
   </sheetData>

</xml_diff>